<commit_message>
Modelo Excel: mescla as linhas de nota (A7, A36 e A51)
As tres notas explicativas passam a ocupar a linha inteira (A:I) com
quebra de texto, em todas as 24 abas mensais.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/IMR Rodocon - 04-23 - Prefeitura Universitaria.xlsx
+++ b/IMR Rodocon - 04-23 - Prefeitura Universitaria.xlsx
@@ -978,7 +978,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -1645,7 +1645,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -1914,7 +1914,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -2059,7 +2059,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -2118,8 +2119,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -2341,7 +2344,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -3016,7 +3019,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -3286,7 +3289,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -3431,7 +3434,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -3490,8 +3494,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -3713,7 +3719,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -4388,7 +4394,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -4658,7 +4664,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -4803,7 +4809,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -4862,8 +4869,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -5085,7 +5094,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -5760,7 +5769,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -6030,7 +6039,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -6175,7 +6184,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -6234,8 +6244,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -6457,7 +6469,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -7132,7 +7144,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -7402,7 +7414,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -7547,7 +7559,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -7606,8 +7619,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -7829,7 +7844,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -8504,7 +8519,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -8774,7 +8789,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -8919,7 +8934,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -8978,8 +8994,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -9201,7 +9219,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -9876,7 +9894,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -10146,7 +10164,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -10291,7 +10309,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -10350,8 +10369,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -10573,7 +10594,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -11248,7 +11269,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -11518,7 +11539,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -11663,7 +11684,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -11722,8 +11744,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -11945,7 +11969,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -12620,7 +12644,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -12890,7 +12914,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -13035,7 +13059,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -13094,8 +13119,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -13317,7 +13344,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -13992,7 +14019,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -14262,7 +14289,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -14407,7 +14434,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -14466,8 +14494,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -14689,7 +14719,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -15364,7 +15394,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -15634,7 +15664,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -15779,7 +15809,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -15838,8 +15869,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -16061,7 +16094,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -16736,7 +16769,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -17006,7 +17039,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -17151,7 +17184,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -17210,8 +17244,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -17433,7 +17469,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -18108,7 +18144,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -18378,7 +18414,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -18523,7 +18559,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -18582,8 +18619,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -18805,7 +18844,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -19480,7 +19519,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -19750,7 +19789,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -19895,7 +19934,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -19954,8 +19994,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -20177,7 +20219,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -20852,7 +20894,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -21122,7 +21164,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -21267,7 +21309,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -21326,8 +21369,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -21549,7 +21594,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -22224,7 +22269,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -22494,7 +22539,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -22639,7 +22684,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -22698,8 +22744,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -22921,7 +22969,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -23596,7 +23644,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -23866,7 +23914,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -24011,7 +24059,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -24070,8 +24119,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -25559,7 +25610,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -26234,7 +26285,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -26504,7 +26555,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -26649,7 +26700,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -26708,8 +26760,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -26931,7 +26985,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -27606,7 +27660,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -27876,7 +27930,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -28021,7 +28075,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -28080,8 +28135,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -28303,7 +28360,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -28978,7 +29035,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -29248,7 +29305,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -29393,7 +29450,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -29452,8 +29510,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -29675,7 +29735,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -30350,7 +30410,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -30620,7 +30680,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -30765,7 +30825,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -30824,8 +30885,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -31047,7 +31110,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -31722,7 +31785,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -31992,7 +32055,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -32137,7 +32200,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -32196,8 +32260,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -32419,7 +32485,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -33094,7 +33160,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -33364,7 +33430,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -33509,7 +33575,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -33568,8 +33635,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>
@@ -33791,7 +33860,7 @@
       <c r="H6" s="7" t="n"/>
       <c r="I6" s="7" t="n"/>
     </row>
-    <row r="7">
+    <row r="7" ht="14" customHeight="1">
       <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Preencha as células em amarelo. Pontuação, nota e valores são calculados automaticamente.</t>
@@ -34466,7 +34535,7 @@
       </c>
       <c r="I35" s="34" t="n"/>
     </row>
-    <row r="36">
+    <row r="36" ht="28" customHeight="1">
       <c r="A36" s="10" t="inlineStr">
         <is>
           <t>Retido = qtde contratada × valor estimado unitário · Total = reembolsos aprovados × valor por dependente · Saldo = saldo do mês anterior + retido − total.</t>
@@ -34736,7 +34805,7 @@
         <v/>
       </c>
     </row>
-    <row r="51">
+    <row r="51" ht="14" customHeight="1">
       <c r="A51" s="10" t="inlineStr">
         <is>
           <t>Qtde Faturada = QTD TOTAL da planilha orçamentária · Valor Unit. Faturado = valor dos serviços ÷ Qtde Faturada.</t>
@@ -34881,7 +34950,8 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="1" password="C71F"/>
-  <mergeCells count="69">
+  <mergeCells count="72">
+    <mergeCell ref="A7:I7"/>
     <mergeCell ref="G21:H21"/>
     <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
@@ -34940,8 +35010,10 @@
     <mergeCell ref="A35:B35"/>
     <mergeCell ref="B49:F49"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A51:I51"/>
     <mergeCell ref="A45:C45"/>
     <mergeCell ref="B15:F15"/>
+    <mergeCell ref="A36:I36"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A1:I1"/>
     <mergeCell ref="A28:B28"/>

</xml_diff>